<commit_message>
[add] solucio headers amb boostrap i cataleg productes
</commit_message>
<xml_diff>
--- a/productes.xlsx
+++ b/productes.xlsx
@@ -20,24 +20,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
-  <si>
-    <t xml:space="preserve">SKU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descripcio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">img</t>
-  </si>
-  <si>
-    <t xml:space="preserve">preu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">estoc</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t xml:space="preserve">sku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock</t>
   </si>
   <si>
     <t xml:space="preserve">A001</t>
@@ -49,9 +46,6 @@
     <t xml:space="preserve">Anell de plata minimalista amb disseny orgànic.</t>
   </si>
   <si>
-    <t xml:space="preserve">./contenido/image_anell.png</t>
-  </si>
-  <si>
     <t xml:space="preserve">29.99</t>
   </si>
   <si>
@@ -64,9 +58,6 @@
     <t xml:space="preserve">Collaret d'acer inoxidable amb penjoll de creu.</t>
   </si>
   <si>
-    <t xml:space="preserve">./contenido/image.png</t>
-  </si>
-  <si>
     <t xml:space="preserve">45.50</t>
   </si>
   <si>
@@ -77,9 +68,6 @@
   </si>
   <si>
     <t xml:space="preserve">Arracades de cèrcol petites d'estil clàssic.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">./contenido/arracades.png</t>
   </si>
   <si>
     <t xml:space="preserve">19.95</t>
@@ -92,7 +80,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -119,6 +107,11 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -176,11 +169,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -317,7 +310,7 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -326,72 +319,60 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="E2" s="2" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="1" t="n">
+      <c r="E3" s="1" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="F4" s="1" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G15" s="3"/>
+      <c r="G15" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K17" s="4"/>

</xml_diff>